<commit_message>
upgrade maven generator to 0.5.2
</commit_message>
<xml_diff>
--- a/src/main/resources/be/vlaanderen/bodemenondergrond/data/id/conceptscheme/materiaalklasse/materiaalklasse.xlsx
+++ b/src/main/resources/be/vlaanderen/bodemenondergrond/data/id/conceptscheme/materiaalklasse/materiaalklasse.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P40"/>
+  <dimension ref="A1:O39"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -410,75 +410,72 @@
         <v>dc\.identifier</v>
       </c>
       <c r="D1" t="str">
+        <v>broader</v>
+      </c>
+      <c r="E1" t="str">
+        <v>broaderTransitive</v>
+      </c>
+      <c r="F1" t="str">
         <v>inScheme</v>
       </c>
-      <c r="E1" t="str">
-        <v>member</v>
-      </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>notation</v>
       </c>
-      <c r="G1" t="str">
+      <c r="H1" t="str">
         <v>prefLabel</v>
       </c>
-      <c r="H1" t="str">
-        <v>broader</v>
-      </c>
       <c r="I1" t="str">
-        <v>broaderTransitive</v>
+        <v>semanticRelation</v>
       </c>
       <c r="J1" t="str">
-        <v>semanticRelation</v>
+        <v>topConceptOf</v>
       </c>
       <c r="K1" t="str">
-        <v>topConceptOf</v>
+        <v>narrower</v>
       </c>
       <c r="L1" t="str">
-        <v>narrower</v>
+        <v>narrowerTransitive</v>
       </c>
       <c r="M1" t="str">
-        <v>narrowerTransitive</v>
+        <v>definition</v>
       </c>
       <c r="N1" t="str">
-        <v>definition</v>
+        <v>hasTopConcept</v>
       </c>
       <c r="O1" t="str">
-        <v>hasTopConcept</v>
-      </c>
-      <c r="P1" t="str">
         <v>note</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/collection/materiaalklasse/materiaalklasses</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/afvalwater</v>
       </c>
       <c r="B2" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Collection</v>
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C2" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.collection.materiaalklasse.materiaalklasses</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.afvalwater</v>
       </c>
       <c r="D2" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="E2" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/afvalwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bemalingswater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodem|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemlucht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemvocht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/depositie|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/drinkwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/effluent|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eieren|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eluaat|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/fruit|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/gftafval|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/groenten|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/grondwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/hardgesteente|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/koelwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/melk|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/migratie|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/oppervlaktewater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/puurproduct|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/regenwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/schelpdieren|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/sediment|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/strooisel|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vilt|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/waterbodem|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zwevendestof</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="F2" t="str">
-        <v>materiaalklasses</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G2" t="str">
-        <v>Collectie van materiaalklasses.</v>
+        <v>afvalwater</v>
       </c>
       <c r="H2" t="str">
-        <v>null</v>
+        <v>Afvalwater</v>
       </c>
       <c r="I2" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="J2" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K2" t="str">
         <v>null</v>
@@ -493,48 +490,45 @@
         <v>null</v>
       </c>
       <c r="O2" t="str">
-        <v>null</v>
-      </c>
-      <c r="P2" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/afvalwater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
       </c>
       <c r="B3" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C3" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.afvalwater</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.antropogeneobjecten</v>
       </c>
       <c r="D3" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="E3" t="str">
         <v>null</v>
       </c>
       <c r="F3" t="str">
-        <v>afvalwater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G3" t="str">
-        <v>Afvalwater</v>
+        <v>antropogeneobjecten</v>
       </c>
       <c r="H3" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>Antropogene objecten</v>
       </c>
       <c r="I3" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/puurproduct</v>
       </c>
       <c r="J3" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K3" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/puurproduct</v>
       </c>
       <c r="L3" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/puurproduct</v>
       </c>
       <c r="M3" t="str">
         <v>null</v>
@@ -543,95 +537,89 @@
         <v>null</v>
       </c>
       <c r="O3" t="str">
-        <v>null</v>
-      </c>
-      <c r="P3" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bemalingswater</v>
       </c>
       <c r="B4" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C4" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.antropogeneobjecten</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.bemalingswater</v>
       </c>
       <c r="D4" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="E4" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="F4" t="str">
-        <v>antropogeneobjecten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G4" t="str">
-        <v>Antropogene objecten</v>
+        <v>bemalingswater</v>
       </c>
       <c r="H4" t="str">
-        <v>null</v>
+        <v>Bemalingswater</v>
       </c>
       <c r="I4" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="J4" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/puurproduct</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K4" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L4" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/puurproduct</v>
+        <v>null</v>
       </c>
       <c r="M4" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/puurproduct</v>
+        <v>null</v>
       </c>
       <c r="N4" t="str">
         <v>null</v>
       </c>
       <c r="O4" t="str">
-        <v>null</v>
-      </c>
-      <c r="P4" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bemalingswater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodem</v>
       </c>
       <c r="B5" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C5" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.bemalingswater</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.bodem</v>
       </c>
       <c r="D5" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="E5" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="F5" t="str">
-        <v>bemalingswater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G5" t="str">
-        <v>Bemalingswater</v>
+        <v>bodem</v>
       </c>
       <c r="H5" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>Bodem</v>
       </c>
       <c r="I5" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="J5" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K5" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L5" t="str">
         <v>null</v>
@@ -643,45 +631,42 @@
         <v>null</v>
       </c>
       <c r="O5" t="str">
-        <v>null</v>
-      </c>
-      <c r="P5" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodem</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemlucht</v>
       </c>
       <c r="B6" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C6" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.bodem</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.bodemlucht</v>
       </c>
       <c r="D6" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
       </c>
       <c r="E6" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
       </c>
       <c r="F6" t="str">
-        <v>bodem</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G6" t="str">
-        <v>Bodem</v>
+        <v>bodemlucht</v>
       </c>
       <c r="H6" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>Bodemlucht</v>
       </c>
       <c r="I6" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
       </c>
       <c r="J6" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K6" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L6" t="str">
         <v>null</v>
@@ -693,45 +678,42 @@
         <v>null</v>
       </c>
       <c r="O6" t="str">
-        <v>null</v>
-      </c>
-      <c r="P6" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemlucht</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemvocht</v>
       </c>
       <c r="B7" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C7" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.bodemlucht</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.bodemvocht</v>
       </c>
       <c r="D7" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="E7" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="F7" t="str">
-        <v>bodemlucht</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G7" t="str">
-        <v>Bodemlucht</v>
+        <v>bodemvocht</v>
       </c>
       <c r="H7" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
+        <v>Bodemvocht</v>
       </c>
       <c r="I7" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="J7" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K7" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L7" t="str">
         <v>null</v>
@@ -743,45 +725,42 @@
         <v>null</v>
       </c>
       <c r="O7" t="str">
-        <v>null</v>
-      </c>
-      <c r="P7" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemvocht</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/depositie</v>
       </c>
       <c r="B8" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C8" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.bodemvocht</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.depositie</v>
       </c>
       <c r="D8" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
       </c>
       <c r="E8" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
       </c>
       <c r="F8" t="str">
-        <v>bodemvocht</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G8" t="str">
-        <v>Bodemvocht</v>
+        <v>depositie</v>
       </c>
       <c r="H8" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>Depositie</v>
       </c>
       <c r="I8" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
       </c>
       <c r="J8" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K8" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L8" t="str">
         <v>null</v>
@@ -793,48 +772,45 @@
         <v>null</v>
       </c>
       <c r="O8" t="str">
-        <v>null</v>
-      </c>
-      <c r="P8" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/depositie</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
       </c>
       <c r="B9" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C9" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.depositie</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.dierlijkmateriaal</v>
       </c>
       <c r="D9" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="E9" t="str">
         <v>null</v>
       </c>
       <c r="F9" t="str">
-        <v>depositie</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G9" t="str">
-        <v>Depositie</v>
+        <v>dierlijkmateriaal</v>
       </c>
       <c r="H9" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
+        <v>Dierlijk materiaal</v>
       </c>
       <c r="I9" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eieren|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/melk|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/schelpdieren</v>
       </c>
       <c r="J9" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K9" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eieren|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/melk|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/schelpdieren</v>
       </c>
       <c r="L9" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eieren|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/melk|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/schelpdieren</v>
       </c>
       <c r="M9" t="str">
         <v>null</v>
@@ -843,95 +819,89 @@
         <v>null</v>
       </c>
       <c r="O9" t="str">
-        <v>null</v>
-      </c>
-      <c r="P9" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dnapl</v>
       </c>
       <c r="B10" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C10" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.dierlijkmateriaal</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.dnapl</v>
       </c>
       <c r="D10" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
       </c>
       <c r="E10" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
       </c>
       <c r="F10" t="str">
-        <v>dierlijkmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G10" t="str">
-        <v>Dierlijk materiaal</v>
+        <v>dnapl</v>
       </c>
       <c r="H10" t="str">
-        <v>null</v>
+        <v>Zaklaag (DNAPL)</v>
       </c>
       <c r="I10" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
       </c>
       <c r="J10" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eieren|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/melk|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/schelpdieren</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K10" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L10" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eieren|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/melk|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/schelpdieren</v>
+        <v>null</v>
       </c>
       <c r="M10" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eieren|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/melk|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/schelpdieren</v>
+        <v>null</v>
       </c>
       <c r="N10" t="str">
         <v>null</v>
       </c>
       <c r="O10" t="str">
-        <v>null</v>
-      </c>
-      <c r="P10" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dnapl</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/drinkwater</v>
       </c>
       <c r="B11" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C11" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.dnapl</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.drinkwater</v>
       </c>
       <c r="D11" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="E11" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="F11" t="str">
-        <v>dnapl</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G11" t="str">
-        <v>Zaklaag (DNAPL)</v>
+        <v>drinkwater</v>
       </c>
       <c r="H11" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
+        <v>Drinkwater</v>
       </c>
       <c r="I11" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="J11" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K11" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L11" t="str">
         <v>null</v>
@@ -943,45 +913,42 @@
         <v>null</v>
       </c>
       <c r="O11" t="str">
-        <v>null</v>
-      </c>
-      <c r="P11" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/drinkwater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/effluent</v>
       </c>
       <c r="B12" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C12" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.drinkwater</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.effluent</v>
       </c>
       <c r="D12" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="E12" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="F12" t="str">
-        <v>drinkwater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G12" t="str">
-        <v>Drinkwater</v>
+        <v>effluent</v>
       </c>
       <c r="H12" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>Effluent</v>
       </c>
       <c r="I12" t="str">
         <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="J12" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K12" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L12" t="str">
         <v>null</v>
@@ -993,45 +960,42 @@
         <v>null</v>
       </c>
       <c r="O12" t="str">
-        <v>null</v>
-      </c>
-      <c r="P12" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/effluent</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eieren</v>
       </c>
       <c r="B13" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C13" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.effluent</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.eieren</v>
       </c>
       <c r="D13" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
       </c>
       <c r="E13" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
       </c>
       <c r="F13" t="str">
-        <v>effluent</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G13" t="str">
-        <v>Effluent</v>
+        <v>eieren</v>
       </c>
       <c r="H13" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>Eieren</v>
       </c>
       <c r="I13" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
       </c>
       <c r="J13" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K13" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L13" t="str">
         <v>null</v>
@@ -1043,45 +1007,42 @@
         <v>null</v>
       </c>
       <c r="O13" t="str">
-        <v>null</v>
-      </c>
-      <c r="P13" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eieren</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eluaat</v>
       </c>
       <c r="B14" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C14" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.eieren</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.eluaat</v>
       </c>
       <c r="D14" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="E14" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="F14" t="str">
-        <v>eieren</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G14" t="str">
-        <v>Eieren</v>
+        <v>eluaat</v>
       </c>
       <c r="H14" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
+        <v>Eluaat</v>
       </c>
       <c r="I14" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="J14" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K14" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L14" t="str">
         <v>null</v>
@@ -1093,45 +1054,42 @@
         <v>null</v>
       </c>
       <c r="O14" t="str">
-        <v>null</v>
-      </c>
-      <c r="P14" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eluaat</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/fruit</v>
       </c>
       <c r="B15" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C15" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.eluaat</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.fruit</v>
       </c>
       <c r="D15" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="E15" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="F15" t="str">
-        <v>eluaat</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G15" t="str">
-        <v>Eluaat</v>
+        <v>fruit</v>
       </c>
       <c r="H15" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>Fruit</v>
       </c>
       <c r="I15" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="J15" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K15" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L15" t="str">
         <v>null</v>
@@ -1143,45 +1101,42 @@
         <v>null</v>
       </c>
       <c r="O15" t="str">
-        <v>null</v>
-      </c>
-      <c r="P15" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/fruit</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/gftafval</v>
       </c>
       <c r="B16" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C16" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.fruit</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.gftafval</v>
       </c>
       <c r="D16" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="E16" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="F16" t="str">
-        <v>fruit</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G16" t="str">
-        <v>Fruit</v>
+        <v>gftafval</v>
       </c>
       <c r="H16" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>GFT-afval</v>
       </c>
       <c r="I16" t="str">
         <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="J16" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K16" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L16" t="str">
         <v>null</v>
@@ -1193,45 +1148,42 @@
         <v>null</v>
       </c>
       <c r="O16" t="str">
-        <v>null</v>
-      </c>
-      <c r="P16" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/gftafval</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/groenten</v>
       </c>
       <c r="B17" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C17" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.gftafval</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.groenten</v>
       </c>
       <c r="D17" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="E17" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="F17" t="str">
-        <v>gftafval</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G17" t="str">
-        <v>GFT-afval</v>
+        <v>groenten</v>
       </c>
       <c r="H17" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>Groenten</v>
       </c>
       <c r="I17" t="str">
         <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="J17" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K17" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L17" t="str">
         <v>null</v>
@@ -1243,45 +1195,42 @@
         <v>null</v>
       </c>
       <c r="O17" t="str">
-        <v>null</v>
-      </c>
-      <c r="P17" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/groenten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/grondwater</v>
       </c>
       <c r="B18" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C18" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.groenten</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.grondwater</v>
       </c>
       <c r="D18" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="E18" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="F18" t="str">
-        <v>groenten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G18" t="str">
-        <v>Groenten</v>
+        <v>grondwater</v>
       </c>
       <c r="H18" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>Grondwater</v>
       </c>
       <c r="I18" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="J18" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K18" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L18" t="str">
         <v>null</v>
@@ -1293,45 +1242,42 @@
         <v>null</v>
       </c>
       <c r="O18" t="str">
-        <v>null</v>
-      </c>
-      <c r="P18" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/grondwater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/hardgesteente</v>
       </c>
       <c r="B19" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C19" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.grondwater</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.hardgesteente</v>
       </c>
       <c r="D19" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="E19" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="F19" t="str">
-        <v>grondwater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G19" t="str">
-        <v>Grondwater</v>
+        <v>hardgesteente</v>
       </c>
       <c r="H19" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>Hard gesteente</v>
       </c>
       <c r="I19" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="J19" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K19" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L19" t="str">
         <v>null</v>
@@ -1343,45 +1289,42 @@
         <v>null</v>
       </c>
       <c r="O19" t="str">
-        <v>null</v>
-      </c>
-      <c r="P19" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/hardgesteente</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/koelwater</v>
       </c>
       <c r="B20" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C20" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.hardgesteente</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.koelwater</v>
       </c>
       <c r="D20" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="E20" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="F20" t="str">
-        <v>hardgesteente</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G20" t="str">
-        <v>Hard gesteente</v>
+        <v>koelwater</v>
       </c>
       <c r="H20" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>Koelwater</v>
       </c>
       <c r="I20" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="J20" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K20" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L20" t="str">
         <v>null</v>
@@ -1393,45 +1336,42 @@
         <v>null</v>
       </c>
       <c r="O20" t="str">
-        <v>null</v>
-      </c>
-      <c r="P20" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/koelwater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lnapl</v>
       </c>
       <c r="B21" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C21" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.koelwater</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.lnapl</v>
       </c>
       <c r="D21" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
       </c>
       <c r="E21" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
       </c>
       <c r="F21" t="str">
-        <v>koelwater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G21" t="str">
-        <v>Koelwater</v>
+        <v>lnapl</v>
       </c>
       <c r="H21" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>Drijflaag (LNAPL)</v>
       </c>
       <c r="I21" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
       </c>
       <c r="J21" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K21" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L21" t="str">
         <v>null</v>
@@ -1443,48 +1383,45 @@
         <v>null</v>
       </c>
       <c r="O21" t="str">
-        <v>null</v>
-      </c>
-      <c r="P21" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lnapl</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
       </c>
       <c r="B22" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C22" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.lnapl</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.lucht</v>
       </c>
       <c r="D22" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="E22" t="str">
         <v>null</v>
       </c>
       <c r="F22" t="str">
-        <v>lnapl</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G22" t="str">
-        <v>Drijflaag (LNAPL)</v>
+        <v>lucht</v>
       </c>
       <c r="H22" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
+        <v>Lucht</v>
       </c>
       <c r="I22" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemlucht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/depositie|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zwevendestof</v>
       </c>
       <c r="J22" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K22" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemlucht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/depositie|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zwevendestof</v>
       </c>
       <c r="L22" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemlucht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/depositie|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zwevendestof</v>
       </c>
       <c r="M22" t="str">
         <v>null</v>
@@ -1493,95 +1430,89 @@
         <v>null</v>
       </c>
       <c r="O22" t="str">
-        <v>null</v>
-      </c>
-      <c r="P22" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/melk</v>
       </c>
       <c r="B23" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C23" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.lucht</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.melk</v>
       </c>
       <c r="D23" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
       </c>
       <c r="E23" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
       </c>
       <c r="F23" t="str">
-        <v>lucht</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G23" t="str">
-        <v>Lucht</v>
+        <v>melk</v>
       </c>
       <c r="H23" t="str">
-        <v>null</v>
+        <v>Melk</v>
       </c>
       <c r="I23" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
       </c>
       <c r="J23" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemlucht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/depositie|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zwevendestof</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K23" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L23" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemlucht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/depositie|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zwevendestof</v>
+        <v>null</v>
       </c>
       <c r="M23" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemlucht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/depositie|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zwevendestof</v>
+        <v>null</v>
       </c>
       <c r="N23" t="str">
         <v>null</v>
       </c>
       <c r="O23" t="str">
-        <v>null</v>
-      </c>
-      <c r="P23" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/melk</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/migratie</v>
       </c>
       <c r="B24" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C24" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.melk</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.migratie</v>
       </c>
       <c r="D24" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="E24" t="str">
         <v>null</v>
       </c>
       <c r="F24" t="str">
-        <v>melk</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G24" t="str">
-        <v>Melk</v>
+        <v>migratie</v>
       </c>
       <c r="H24" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
+        <v>Migratie</v>
       </c>
       <c r="I24" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
+        <v>null</v>
       </c>
       <c r="J24" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K24" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L24" t="str">
         <v>null</v>
@@ -1593,45 +1524,42 @@
         <v>null</v>
       </c>
       <c r="O24" t="str">
-        <v>null</v>
-      </c>
-      <c r="P24" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/migratie</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/oppervlaktewater</v>
       </c>
       <c r="B25" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C25" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.migratie</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.oppervlaktewater</v>
       </c>
       <c r="D25" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="E25" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="F25" t="str">
-        <v>migratie</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G25" t="str">
-        <v>Migratie</v>
+        <v>oppervlaktewater</v>
       </c>
       <c r="H25" t="str">
-        <v>null</v>
+        <v>Oppervlaktewater</v>
       </c>
       <c r="I25" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="J25" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K25" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L25" t="str">
         <v>null</v>
@@ -1643,48 +1571,45 @@
         <v>null</v>
       </c>
       <c r="O25" t="str">
-        <v>null</v>
-      </c>
-      <c r="P25" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/oppervlaktewater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="B26" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C26" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.oppervlaktewater</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.plantaardigmateriaal</v>
       </c>
       <c r="D26" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="E26" t="str">
         <v>null</v>
       </c>
       <c r="F26" t="str">
-        <v>oppervlaktewater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G26" t="str">
-        <v>Oppervlaktewater</v>
+        <v>plantaardigmateriaal</v>
       </c>
       <c r="H26" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>Plantaardig materiaal</v>
       </c>
       <c r="I26" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/fruit|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/gftafval|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/groenten|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/strooisel|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vilt</v>
       </c>
       <c r="J26" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K26" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/fruit|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/gftafval|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/groenten|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/strooisel|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vilt</v>
       </c>
       <c r="L26" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/fruit|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/gftafval|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/groenten|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/strooisel|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vilt</v>
       </c>
       <c r="M26" t="str">
         <v>null</v>
@@ -1693,95 +1618,89 @@
         <v>null</v>
       </c>
       <c r="O26" t="str">
-        <v>null</v>
-      </c>
-      <c r="P26" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/puurproduct</v>
       </c>
       <c r="B27" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C27" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.plantaardigmateriaal</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.puurproduct</v>
       </c>
       <c r="D27" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
       </c>
       <c r="E27" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
       </c>
       <c r="F27" t="str">
-        <v>plantaardigmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G27" t="str">
-        <v>Plantaardig materiaal</v>
+        <v>puurproduct</v>
       </c>
       <c r="H27" t="str">
-        <v>null</v>
+        <v>Puur product</v>
       </c>
       <c r="I27" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
       </c>
       <c r="J27" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/fruit|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/gftafval|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/groenten|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/strooisel|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vilt</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K27" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L27" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/fruit|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/gftafval|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/groenten|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/strooisel|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vilt</v>
+        <v>null</v>
       </c>
       <c r="M27" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/fruit|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/gftafval|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/groenten|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/strooisel|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vilt</v>
+        <v>null</v>
       </c>
       <c r="N27" t="str">
         <v>null</v>
       </c>
       <c r="O27" t="str">
-        <v>null</v>
-      </c>
-      <c r="P27" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/puurproduct</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/regenwater</v>
       </c>
       <c r="B28" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C28" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.puurproduct</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.regenwater</v>
       </c>
       <c r="D28" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="E28" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="F28" t="str">
-        <v>puurproduct</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G28" t="str">
-        <v>Puur product</v>
+        <v>regenwater</v>
       </c>
       <c r="H28" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
+        <v>Regenwater</v>
       </c>
       <c r="I28" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="J28" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K28" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L28" t="str">
         <v>null</v>
@@ -1793,45 +1712,42 @@
         <v>null</v>
       </c>
       <c r="O28" t="str">
-        <v>null</v>
-      </c>
-      <c r="P28" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/regenwater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/schelpdieren</v>
       </c>
       <c r="B29" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C29" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.regenwater</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.schelpdieren</v>
       </c>
       <c r="D29" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
       </c>
       <c r="E29" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
       </c>
       <c r="F29" t="str">
-        <v>regenwater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G29" t="str">
-        <v>Regenwater</v>
+        <v>schelpdieren</v>
       </c>
       <c r="H29" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>Schelpdieren</v>
       </c>
       <c r="I29" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
       </c>
       <c r="J29" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K29" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L29" t="str">
         <v>null</v>
@@ -1843,45 +1759,42 @@
         <v>null</v>
       </c>
       <c r="O29" t="str">
-        <v>null</v>
-      </c>
-      <c r="P29" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/schelpdieren</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/sediment</v>
       </c>
       <c r="B30" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C30" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.schelpdieren</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.sediment</v>
       </c>
       <c r="D30" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="E30" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="F30" t="str">
-        <v>schelpdieren</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G30" t="str">
-        <v>Schelpdieren</v>
+        <v>sediment</v>
       </c>
       <c r="H30" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
+        <v>Sediment</v>
       </c>
       <c r="I30" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="J30" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K30" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L30" t="str">
         <v>null</v>
@@ -1893,45 +1806,42 @@
         <v>null</v>
       </c>
       <c r="O30" t="str">
-        <v>null</v>
-      </c>
-      <c r="P30" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/sediment</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/strooisel</v>
       </c>
       <c r="B31" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C31" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.sediment</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.strooisel</v>
       </c>
       <c r="D31" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="E31" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="F31" t="str">
-        <v>sediment</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G31" t="str">
-        <v>Sediment</v>
+        <v>strooisel</v>
       </c>
       <c r="H31" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>Strooisel</v>
       </c>
       <c r="I31" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="J31" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K31" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L31" t="str">
         <v>null</v>
@@ -1943,48 +1853,45 @@
         <v>null</v>
       </c>
       <c r="O31" t="str">
-        <v>null</v>
-      </c>
-      <c r="P31" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/strooisel</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="B32" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C32" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.strooisel</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.vastdeelvdaarde</v>
       </c>
       <c r="D32" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="E32" t="str">
         <v>null</v>
       </c>
       <c r="F32" t="str">
-        <v>strooisel</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G32" t="str">
-        <v>Strooisel</v>
+        <v>vastdeelvdaarde</v>
       </c>
       <c r="H32" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>Vaste deel van de aarde</v>
       </c>
       <c r="I32" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodem|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eluaat|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/hardgesteente|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/sediment|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/waterbodem</v>
       </c>
       <c r="J32" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K32" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodem|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eluaat|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/hardgesteente|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/sediment|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/waterbodem</v>
       </c>
       <c r="L32" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodem|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eluaat|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/hardgesteente|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/sediment|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/waterbodem</v>
       </c>
       <c r="M32" t="str">
         <v>null</v>
@@ -1993,98 +1900,92 @@
         <v>null</v>
       </c>
       <c r="O32" t="str">
-        <v>null</v>
-      </c>
-      <c r="P32" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vilt</v>
       </c>
       <c r="B33" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C33" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.vastdeelvdaarde</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.vilt</v>
       </c>
       <c r="D33" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="E33" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="F33" t="str">
-        <v>vastdeelvdaarde</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G33" t="str">
-        <v>Vaste deel van de aarde</v>
+        <v>vilt</v>
       </c>
       <c r="H33" t="str">
-        <v>null</v>
+        <v>Vilt</v>
       </c>
       <c r="I33" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
       </c>
       <c r="J33" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodem|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eluaat|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/hardgesteente|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/sediment|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/waterbodem</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K33" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L33" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodem|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eluaat|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/hardgesteente|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/sediment|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/waterbodem</v>
+        <v>null</v>
       </c>
       <c r="M33" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodem|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eluaat|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/hardgesteente|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/sediment|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/waterbodem</v>
+        <v>null</v>
       </c>
       <c r="N33" t="str">
         <v>null</v>
       </c>
       <c r="O33" t="str">
-        <v>null</v>
-      </c>
-      <c r="P33" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vilt</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
       </c>
       <c r="B34" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C34" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.vilt</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.water</v>
       </c>
       <c r="D34" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="E34" t="str">
         <v>null</v>
       </c>
       <c r="F34" t="str">
-        <v>vilt</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G34" t="str">
-        <v>Vilt</v>
+        <v>water</v>
       </c>
       <c r="H34" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>Water</v>
       </c>
       <c r="I34" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/afvalwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bemalingswater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemvocht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/drinkwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/effluent|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/grondwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/koelwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/oppervlaktewater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/regenwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
       </c>
       <c r="J34" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K34" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/afvalwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bemalingswater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemvocht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/drinkwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/effluent|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/grondwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/koelwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/oppervlaktewater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/regenwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
       </c>
       <c r="L34" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/afvalwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bemalingswater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemvocht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/drinkwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/effluent|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/grondwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/koelwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/oppervlaktewater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/regenwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
       </c>
       <c r="M34" t="str">
         <v>null</v>
@@ -2093,95 +1994,89 @@
         <v>null</v>
       </c>
       <c r="O34" t="str">
-        <v>null</v>
-      </c>
-      <c r="P34" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/waterbodem</v>
       </c>
       <c r="B35" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C35" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.water</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.waterbodem</v>
       </c>
       <c r="D35" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="E35" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="F35" t="str">
-        <v>water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G35" t="str">
-        <v>Water</v>
+        <v>waterbodem</v>
       </c>
       <c r="H35" t="str">
-        <v>null</v>
+        <v>Waterbodem</v>
       </c>
       <c r="I35" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
       </c>
       <c r="J35" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/afvalwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bemalingswater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemvocht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/drinkwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/effluent|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/grondwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/koelwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/oppervlaktewater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/regenwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K35" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L35" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/afvalwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bemalingswater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemvocht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/drinkwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/effluent|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/grondwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/koelwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/oppervlaktewater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/regenwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
+        <v>null</v>
       </c>
       <c r="M35" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/afvalwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bemalingswater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemvocht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/drinkwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/effluent|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/grondwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/koelwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/oppervlaktewater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/regenwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
+        <v>null</v>
       </c>
       <c r="N35" t="str">
         <v>null</v>
       </c>
       <c r="O35" t="str">
-        <v>null</v>
-      </c>
-      <c r="P35" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/waterbodem</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim</v>
       </c>
       <c r="B36" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C36" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.waterbodem</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.zeeschuim</v>
       </c>
       <c r="D36" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
       </c>
       <c r="E36" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
       </c>
       <c r="F36" t="str">
-        <v>waterbodem</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G36" t="str">
-        <v>Waterbodem</v>
+        <v>zeeschuim</v>
       </c>
       <c r="H36" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>Zeeschuim</v>
       </c>
       <c r="I36" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
       </c>
       <c r="J36" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K36" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L36" t="str">
         <v>null</v>
@@ -2193,48 +2088,45 @@
         <v>null</v>
       </c>
       <c r="O36" t="str">
-        <v>null</v>
-      </c>
-      <c r="P36" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
+      </c>
+      <c r="B37" t="str">
+        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+      </c>
+      <c r="C37" t="str">
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.zeewater</v>
+      </c>
+      <c r="D37" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+      </c>
+      <c r="E37" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+      </c>
+      <c r="F37" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+      </c>
+      <c r="G37" t="str">
+        <v>zeewater</v>
+      </c>
+      <c r="H37" t="str">
+        <v>Zeewater</v>
+      </c>
+      <c r="I37" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim</v>
+      </c>
+      <c r="J37" t="str">
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+      </c>
+      <c r="K37" t="str">
         <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim</v>
       </c>
-      <c r="B37" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
-      </c>
-      <c r="C37" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.zeeschuim</v>
-      </c>
-      <c r="D37" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
-      </c>
-      <c r="E37" t="str">
-        <v>null</v>
-      </c>
-      <c r="F37" t="str">
-        <v>zeeschuim</v>
-      </c>
-      <c r="G37" t="str">
-        <v>Zeeschuim</v>
-      </c>
-      <c r="H37" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
-      </c>
-      <c r="I37" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
-      </c>
-      <c r="J37" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
-      </c>
-      <c r="K37" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
-      </c>
       <c r="L37" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim</v>
       </c>
       <c r="M37" t="str">
         <v>null</v>
@@ -2243,165 +2135,106 @@
         <v>null</v>
       </c>
       <c r="O37" t="str">
-        <v>null</v>
-      </c>
-      <c r="P37" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zwevendestof</v>
       </c>
       <c r="B38" t="str">
         <v>http://www.w3.org/2004/02/skos/core#Concept</v>
       </c>
       <c r="C38" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.zeewater</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.zwevendestof</v>
       </c>
       <c r="D38" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
       </c>
       <c r="E38" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
       </c>
       <c r="F38" t="str">
-        <v>zeewater</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="G38" t="str">
-        <v>Zeewater</v>
+        <v>zwevendestof</v>
       </c>
       <c r="H38" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>Zwevende stof</v>
       </c>
       <c r="I38" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
       </c>
       <c r="J38" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="K38" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L38" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim</v>
+        <v>null</v>
       </c>
       <c r="M38" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim</v>
+        <v>null</v>
       </c>
       <c r="N38" t="str">
         <v>null</v>
       </c>
       <c r="O38" t="str">
-        <v>null</v>
-      </c>
-      <c r="P38" t="str">
         <v>null</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zwevendestof</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
       </c>
       <c r="B39" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#Concept</v>
+        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
       </c>
       <c r="C39" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.concept.materiaalklasse.zwevendestof</v>
+        <v>be.vlaanderen.bodemenondergrond.data.id.conceptscheme.materiaalklasse</v>
       </c>
       <c r="D39" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="E39" t="str">
         <v>null</v>
       </c>
       <c r="F39" t="str">
-        <v>zwevendestof</v>
+        <v>null</v>
       </c>
       <c r="G39" t="str">
-        <v>Zwevende stof</v>
+        <v>materiaalklasse</v>
       </c>
       <c r="H39" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
+        <v>Codelijst materiaalklasse.</v>
       </c>
       <c r="I39" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
+        <v>null</v>
       </c>
       <c r="J39" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht</v>
+        <v>null</v>
       </c>
       <c r="K39" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
+        <v>null</v>
       </c>
       <c r="L39" t="str">
         <v>null</v>
       </c>
       <c r="M39" t="str">
-        <v>null</v>
+        <v>Aard van de Bemonstering.</v>
       </c>
       <c r="N39" t="str">
-        <v>null</v>
+        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/afvalwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bemalingswater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodem|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemlucht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemvocht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/depositie|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/drinkwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/effluent|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eieren|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eluaat|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/fruit|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/gftafval|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/groenten|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/grondwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/hardgesteente|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/koelwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/melk|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/migratie|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/oppervlaktewater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/puurproduct|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/regenwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/schelpdieren|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/sediment|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/strooisel|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vilt|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/waterbodem|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zwevendestof</v>
       </c>
       <c r="O39" t="str">
-        <v>null</v>
-      </c>
-      <c r="P39" t="str">
-        <v>null</v>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/conceptscheme/materiaalklasse</v>
-      </c>
-      <c r="B40" t="str">
-        <v>http://www.w3.org/2004/02/skos/core#ConceptScheme</v>
-      </c>
-      <c r="C40" t="str">
-        <v>be.vlaanderen.bodemenondergrond.data.id.conceptscheme.materiaalklasse</v>
-      </c>
-      <c r="D40" t="str">
-        <v>null</v>
-      </c>
-      <c r="E40" t="str">
-        <v>null</v>
-      </c>
-      <c r="F40" t="str">
-        <v>materiaalklasse</v>
-      </c>
-      <c r="G40" t="str">
-        <v>Codelijst materiaalklasse.</v>
-      </c>
-      <c r="H40" t="str">
-        <v>null</v>
-      </c>
-      <c r="I40" t="str">
-        <v>null</v>
-      </c>
-      <c r="J40" t="str">
-        <v>null</v>
-      </c>
-      <c r="K40" t="str">
-        <v>null</v>
-      </c>
-      <c r="L40" t="str">
-        <v>null</v>
-      </c>
-      <c r="M40" t="str">
-        <v>null</v>
-      </c>
-      <c r="N40" t="str">
-        <v>Aard van de Bemonstering.</v>
-      </c>
-      <c r="O40" t="str">
-        <v>https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/afvalwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/antropogeneobjecten|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bemalingswater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodem|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemlucht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/bodemvocht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/depositie|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dierlijkmateriaal|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/dnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/drinkwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/effluent|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eieren|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/eluaat|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/fruit|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/gftafval|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/groenten|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/grondwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/hardgesteente|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/koelwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lnapl|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/lucht|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/melk|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/migratie|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/oppervlaktewater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/plantaardigmateriaal|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/puurproduct|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/regenwater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/schelpdieren|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/sediment|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/strooisel|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vastdeelvdaarde|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/vilt|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/water|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/waterbodem|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeeschuim|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zeewater|https://data.bodemenondergrond.vlaanderen.be/id/concept/materiaalklasse/zwevendestof</v>
-      </c>
-      <c r="P40" t="str">
         <v>Aard van de Bemonstering.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P40"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:O39"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>